<commit_message>
Animate receipt bottom sheet and fix compare-drawer close button
Bottom sheet and compare drawer now slide in with a real enter
transition instead of appearing instantly. Also fixes the drawer's
close button being unclickable on wide desktop viewports: the modal
backdrop's fixed+z-50 wrapper created its own stacking context, which
capped the z-60 drawer below the z-60 ad rail sitting at the page root.
Raised the backdrop to z-70 so the whole modal group paints above it.
</commit_message>
<xml_diff>
--- a/supabase/parts_db_rebuild.xlsx
+++ b/supabase/parts_db_rebuild.xlsx
@@ -2668,7 +2668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2682,6 +2682,8 @@
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2740,6 +2742,16 @@
           <t>extra</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>m2_pcie_top</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>m2_pcie_verified</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2784,6 +2796,14 @@
           <t>DDR5</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2833,6 +2853,14 @@
           <t>{"pcie_x1_slots": 2}</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2874,6 +2902,14 @@
           <t>DDR5</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2918,6 +2954,14 @@
           <t>DDR5</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2959,6 +3003,14 @@
           <t>DDR5</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3000,6 +3052,14 @@
           <t>DDR4</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3046,6 +3106,14 @@
           <t>{"pcie_note": "자료마다 표기 다름, 재확인 필요"}</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3095,6 +3163,14 @@
           <t>{"pcie_x1_slots": 1}</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3144,6 +3220,14 @@
           <t>{"pcie_x1_slots": 1}</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3185,6 +3269,14 @@
           <t>DDR5</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3231,6 +3323,14 @@
           <t>{"pcie_x4_slots": 1}</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3280,6 +3380,14 @@
           <t>{"pcie_x1_slots": 1}</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3326,6 +3434,14 @@
           <t>{"pcie_x4_slots": 1}</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3375,6 +3491,14 @@
           <t>{"note": "확장슬롯 1개뿐, 추가 확장카드 불가"}</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3421,6 +3545,14 @@
           <t>{"pcie_x1_slots": 1}</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3467,6 +3599,14 @@
           <t>{"pcie_x4_slots": 2, "pcie_x1_slots": 1}</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3516,6 +3656,14 @@
           <t>{"pcie_x1_slots": 1, "pcie_x4_slots": 1}</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3565,6 +3713,14 @@
           <t>{"pcie_x1_slots": 1, "note": "2번째 PCIex16 전기적 대역폭 재확인 필요"}</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3614,6 +3770,14 @@
           <t>{"pcie_x1_slots": 1, "note": "CrossFireX 지원, 2번째 슬롯 대역폭 재확인 필요"}</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3663,6 +3827,14 @@
           <t>{"pcie_x1_slots": 2}</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>PCIe3.0x4</t>
+        </is>
+      </c>
+      <c r="M21" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3712,6 +3884,14 @@
           <t>{"pcie_x1_slots": 1}</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>PCIe3.0x4</t>
+        </is>
+      </c>
+      <c r="M22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3758,6 +3938,14 @@
           <t>{"pcie_note": "PCIe4.0, PCIe3.0"}</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M23" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3804,6 +3992,14 @@
           <t>{"pcie_note": "PCIe4.0, PCIe3.0"}</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M24" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3850,6 +4046,14 @@
           <t>{"pcie_note": "PCIe5.0, PCIe4.0"}</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3896,6 +4100,14 @@
           <t>{"pcie_note": "PCIe4.0, PCIe3.0"}</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M26" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3942,6 +4154,14 @@
           <t>{"pcie_note": "PCIe5.0, PCIe4.0"}</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M27" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3988,6 +4208,14 @@
           <t>{"pcie_note": "PCIe5.0, PCIe4.0"}</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M28" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4034,6 +4262,14 @@
           <t>{"pcie_note": "PCIe5.0, PCIe4.0"}</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4080,6 +4316,14 @@
           <t>{"pcie_note": "PCIe5.0, PCIe3.0"}</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4126,6 +4370,14 @@
           <t>{"pcie_note": "PCIe4.0, PCIe3.0"}</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M31" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4172,6 +4424,14 @@
           <t>{"pcie_note": "PCIe5.0, PCIe4.0"}</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4218,6 +4478,14 @@
           <t>{"pcie_note": "PCIe5.0, PCIe4.0"}</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M33" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4264,6 +4532,14 @@
           <t>{"pcie_note": "PCIe4.0, PCIe3.0(x1 슬롯 2개), PCIex16 개수 스펙 미기재라 VGA연결단자 기준 1개로 추정"}</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M34" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4310,6 +4586,14 @@
           <t>{"pcie_note": "PCIe4.0, PCIe3.0"}</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M35" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4356,6 +4640,14 @@
           <t>{"pcie_note": "PCIe5.0, PCIe4.0"}</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4402,6 +4694,14 @@
           <t>{"pcie_note": "PCIe4.0, PCIe3.0"}</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M37" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4448,6 +4748,14 @@
           <t>{"pcie_note": "PCIe4.0, PCIe3.0"}</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M38" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4496,6 +4804,470 @@
         <is>
           <t>{"power_stages": "16+2+1", "m2_slots": 4, "wifi": "WiFi7(MediaTek MT7925)", "usb4_ports": 2, "note": "물리 PCIe x16 슬롯 총 2개: 1번=PCIe5.0x16(라이젠9000/7000 x16모드, 8000시리즈는 PCIe4.0 x8/x4), 2번=PCIe4.0x16 규격(전기적 x4). 초안의 total_slots=3은 오검증, 공식스펙+Newegg 확인 결과 2개로 정정.", "edition": "hatsune_miku", "source": "rog.asus.com,newegg,danawa"}</t>
         </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>mb-39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ASUS TUF GAMING Z790-PLUS WIFI D4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>LGA1700</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Z790</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>305</v>
+      </c>
+      <c r="G40" t="n">
+        <v>244</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>{"power_stages": "16+1", "m2_slots": 4, "wifi": "WiFi6", "note": "슬롯구성 1xPCIe5.0x16 + 1xPCIe4.0x16(전기적x4) + 별도 PCIe4.0x4/PCIe3.0x1 -- x16 총슬롯 2개만 카운트", "source": "asus.com,walmart"}</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>mb-40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ASRock B860M Pro RS WiFi</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>LGA1851</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>B860</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>M-ATX</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>244</v>
+      </c>
+      <c r="G41" t="n">
+        <v>244</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DDR5</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>{"power_stages": "10+1+1+1+1 Dr.MOS", "wifi": "WiFi6E", "note": "PCIe5.0x16 물리슬롯 1개 + 별도 PCIe4.0x4(짧은 슬롯, x16 총슬롯 카운트에서 제외)", "source": "asrock.com,newegg,amazon"}</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>mb-41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ASRock H810M-X</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>LGA1851</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>H810</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>M-ATX</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>244</v>
+      </c>
+      <c r="G42" t="n">
+        <v>244</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DDR5</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>{"note": "보급형 보드, PCIe4.0 x16 슬롯 1개, WiFi 미탑재", "source": "asrock.com,amazon"}</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>mb-42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>GIGABYTE B760 GAMING X AX DDR4</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>LGA1700</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>B760</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>305</v>
+      </c>
+      <c r="G43" t="n">
+        <v>244</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" t="n">
+        <v>3</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>{"power_stages": "8+1+1 Hybrid", "wifi": "WiFi6E", "note": "물리 PCIe x16 슬롯 3개(1번만 전체 대역폭), DDR5 버전(B760 GAMING X AX)과 별도 모델", "source": "gigabyte.com,amazon"}</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>mb-43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ASUS PRIME H610M-K D4</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>LGA1700</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>H610</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>M-ATX</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>244</v>
+      </c>
+      <c r="G44" t="n">
+        <v>244</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>{"note": "DIMM 2슬롯(최대128GB 아님, 실제 64GB), M.2 슬롯 1개뿐(SATA6G_4와 대역폭 공유)", "source": "asus.com,amazon"}</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>PCIe3.0x4</t>
+        </is>
+      </c>
+      <c r="M44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>mb-44</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MSI PRO Z890-A WIFI</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>LGA1851</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Z890</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>305</v>
+      </c>
+      <c r="G45" t="n">
+        <v>244</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1</v>
+      </c>
+      <c r="I45" t="n">
+        <v>2</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>DDR5</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>{"power_stages": "90A SPS VRM", "wifi": "WiFi7", "note": "슬롯구성 1xPCIe5.0x16 + 1xPCIe4.0x16", "source": "msi.com,newegg,amazon"}</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>mb-45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ASUS PRIME Z790-P WIFI D4</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>LGA1700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Z790</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>305</v>
+      </c>
+      <c r="G46" t="n">
+        <v>244</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" t="n">
+        <v>4</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>{"power_stages": "14+1 DrMOS", "wifi": "WiFi6", "m2_slots": 3, "note": "M.2 3개 전부 PCIe4.0x4 (M.2_3은 SATA겸용). x16 물리슬롯 4개 중 1개만 전체대역폭", "source": "asus.com,amazon"}</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>mb-46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>GIGABYTE B860 GAMING X WIFI6E</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>LGA1851</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>B860</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>305</v>
+      </c>
+      <c r="G47" t="n">
+        <v>244</v>
+      </c>
+      <c r="H47" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>DDR5</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>{"power_stages": "12+1+2+1 Phases", "wifi": "WiFi6E", "m2_slots": 3, "note": "M.2 구성 1xPCIe5.0 + 2xPCIe4.0. x16 총슬롯 수는 공식 자료에 명확히 안 나와서 1개(안전값)로 표기, 재확인 권장", "source": "gigabyte.com,amazon"}</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+      <c r="M47" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4509,7 +5281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5310,6 +6082,174 @@
         <is>
           <t>{"capacity_gb": 16}</t>
         </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ram-28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Corsair Vengeance LPX DDR4-3200 CL16 (16GB)</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E29" t="n">
+        <v>31</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ram-29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>G.SKILL Ripjaws V DDR4-3200 CL16 (16GB)</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E30" t="n">
+        <v>42</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ram-30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Kingston FURY Beast DDR4-3200 (16GB)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E31" t="n">
+        <v>34</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>{"note": "높이는 제조사 유통채널 공통 표기치(소수점 단위 공식 datasheet 미확인)"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ram-31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ADATA XPG GAMMIX D30 DDR4-3200 (8GB)</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E32" t="n">
+        <v>34</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>{"note": "높이는 제조사 유통채널 공통 표기치(소수점 단위 공식 datasheet 미확인)"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ram-32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TeamGroup T-Create Classic DDR4-3200 (16GB)</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E33" t="n">
+        <v>34</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>{"note": "JEDEC 표준전압 저프로파일 모델(XMP 오버클럭 아님)"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ram-33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Micron Crucial DDR4-3200 (16GB) 벌크</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>
@@ -10153,7 +11093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11149,6 +12089,116 @@
       <c r="D45" t="inlineStr">
         <is>
           <t>PCIe4.0x4</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ssd-45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Micron Crucial T705 M.2 NVMe (1TB)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>M.2 NVMe</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ssd-46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Micron Crucial T710 M.2 NVMe (2TB)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>M.2 NVMe</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ssd-47</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Kingston FURY Renegade G5 M.2 NVMe (2TB)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>M.2 NVMe</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ssd-48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Western Digital WD_BLACK SN8100 M.2 NVMe (1TB)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>M.2 NVMe</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ssd-49</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Corsair MP700 PRO SE M.2 NVMe (2TB)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>M.2 NVMe</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>PCIe5.0x4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: add 27 more danawa-sourced parts across all 8 categories
Widens option variety per category (budget/high-end CPUs, 8GB/non-XT
GPU variants, X570/DDR5-Z790/A620 boards, SFX/high-wattage PSUs,
Mini-ITX/dual-chamber cases, low-profile/AIO coolers, etc). Also fixes
danawa.py's product-list selector, which broke after a markup change
on danawa's search page.
</commit_message>
<xml_diff>
--- a/supabase/parts_db_rebuild.xlsx
+++ b/supabase/parts_db_rebuild.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2657,6 +2657,311 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>cpu-38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>라이젠5</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>9600</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>그래니트 릿지</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>AM5</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>6C/12T</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="I39" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>6MB/32MB</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>65</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>DDR5-5600</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>{"tdp_max_ppt_w": 88, "has_igpu": true}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>cpu-39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>i9</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>13900K</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>랩터레이크</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>LGA1700</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>24C/32T</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>3</v>
+      </c>
+      <c r="I40" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>32MB/36MB</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>125</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>DDR5-5600/DDR4-3200</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>{"tdp_range_w": "125-253", "has_igpu": true}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>cpu-40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>i5</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>12400</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>엘더레이크</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>LGA1700</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>6C/12T</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I41" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>7.5MB/18MB</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>65</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>DDR4-3200/DDR5-4800</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>{"tdp_range_w": "65-117", "has_igpu": true}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>cpu-41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>i5</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>13500</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>랩터레이크</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>LGA1700</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>14C/20T</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I42" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>11.5MB/24MB</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>65</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>DDR5-4800/DDR4-3200</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>{"tdp_range_w": "65-154", "has_igpu": true}</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>cpu-42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>라이젠3</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>3200G</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>피카소</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>AM4</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>4C/4T</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I43" t="n">
+        <v>4</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2MB/4MB</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>65</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>DDR4-2933</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>{"has_igpu": true, "gpu_model": "Radeon Vega 8"}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2668,7 +2973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5270,6 +5575,177 @@
         <v>1</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>mb-47</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ASUS ROG STRIX X570-E GAMING WIFI II 대원씨티에스</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AM4</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>X570</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>305</v>
+      </c>
+      <c r="G48" t="n">
+        <v>244</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2</v>
+      </c>
+      <c r="I48" t="n">
+        <v>3</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>{"pcie_x1_slots": 2, "m2_slots": 2, "sata_ports": 8, "source": "danawa"}</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>mb-48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>GIGABYTE Z790 AORUS ELITE AX 피씨디렉트</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>LGA1700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Z790</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>305</v>
+      </c>
+      <c r="G49" t="n">
+        <v>244</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" t="n">
+        <v>3</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>DDR5</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>{"pcie_x4_slots": 2, "m2_slots": 4, "note": "23년 11월 리비전 이후 전원부 70→90A, PCB/무선모듈 변경, 구매시 리비전 확인", "source": "danawa"}</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>mb-49</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ASRock A620M-HDV/M.2 디앤디컴</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AM5</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>A620</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>M-ATX</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>244</v>
+      </c>
+      <c r="G50" t="n">
+        <v>226</v>
+      </c>
+      <c r="H50" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" t="n">
+        <v>1</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>DDR5</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>{"pcie_x1_slots": 2, "m2_slots": 2, "sata_ports": 2, "source": "danawa"}</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+      <c r="M50" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5281,7 +5757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6252,6 +6728,93 @@
         <v>1.2</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ram-34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>DDR5</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>G.SKILL DDR5-7200 CL34 TRIDENT Z5 RGB J 패키지</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E35" t="n">
+        <v>44</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>{"cl": "34-45-45-115"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ram-35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CORSAIR DDR4-2666 CL16 VENGEANCE LPX 레드</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2666</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>{"cl": "16-18-18-35"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ram-36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DDR5</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>킹스톤 FURY DDR5-5600 CL36 Beast 블랙 코잇</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>5600</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>{"capacity_gb": 32, "cl": "36-38-38"}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6263,7 +6826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8436,6 +8999,156 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>gpu-45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>RTX50</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PALIT 지포스 RTX 5060 Ti DUAL D7 8GB 이엠텍</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>8</v>
+      </c>
+      <c r="E46" t="n">
+        <v>180</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>8핀</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>600</v>
+      </c>
+      <c r="H46" t="n">
+        <v>262.1</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2슬롯(40.1mm)</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>2</v>
+      </c>
+      <c r="K46" t="b">
+        <v>1</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>{"base_mhz": 2407, "boost_mhz": 2572, "pcie": "PCIe5.0x16(at x8)", "stream_processors": 4608, "memory_type": "GDDR7", "source": "danawa"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>gpu-46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>RX9000</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>GIGABYTE 라데온 RX 9060 XT GAMING OC D6 8GB 피씨디렉트</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>8</v>
+      </c>
+      <c r="E47" t="n">
+        <v>160</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>8핀x1</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>450</v>
+      </c>
+      <c r="H47" t="n">
+        <v>281</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>3슬롯(40mm)</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K47" t="b">
+        <v>1</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>{"boost_mhz": 3320, "pcie": "PCIe5.0x16", "stream_processors": 2048, "memory_type": "GDDR6", "source": "danawa"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>gpu-47</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>RX9000</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SAPPHIRE 라데온 RX 9070 PULSE D6 16GB</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>16</v>
+      </c>
+      <c r="E48" t="n">
+        <v>220</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>8핀x2</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>650</v>
+      </c>
+      <c r="H48" t="n">
+        <v>280</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2슬롯(51.5mm)</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" t="b">
+        <v>1</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>{"boost_mhz": 2520, "pcie": "PCIe5.0x16", "stream_processors": 3584, "memory_type": "GDDR6", "source": "danawa"}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8447,7 +9160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9474,6 +10187,115 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>psu-30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Corsair SF750 (SFX, ATX3.1)</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>750</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>플래티넘</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>100</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>ATX3.1</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>SFX</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>{"connectors": "24핀, EPS(4+4)x2, 12VHPWR x1, PCIe8핀x2, SATAx8", "fan_mm": 92, "note": "팬리스모드 지원, 24년 7월 ATX3.0→ATX3.1 인증 추가", "source": "danawa"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>psu-31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>시소닉 PRIME TITANIUM TX-1600 풀모듈러 ATX3.1</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1600</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>티타늄</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>210</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ATX3.1</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>{"connectors": "24핀, EPS(4+4)x3, 12V2x6 x2, PCIe8핀x6, SATAx16", "fan_mm": 135, "warranty_years": 12, "source": "danawa"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>psu-32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>마이크로닉스 Classic II 풀체인지 600W 80PLUS브론즈 ATX3.1</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>600</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>브론즈</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>140</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ATX3.1</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9485,7 +10307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11082,6 +11904,193 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>case-32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Fractal Design Define 7</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>미들타워</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>E-ATX;ATX;M-ATX;Mini-ITX</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>470</v>
+      </c>
+      <c r="F33" t="n">
+        <v>185</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>표준-ATX</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>하단후면</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>case-33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SilverStone SUGO SST-SG13B-C</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>미니ITX</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Mini-ITX</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>270</v>
+      </c>
+      <c r="F34" t="n">
+        <v>61</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>표준-ATX</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>상단</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>case-34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>쿨러마스터 MasterBox TD500 Mesh V2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>미들타워</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>E-ATX;ATX;M-ATX;Mini-ITX;SSI-CEB</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>410</v>
+      </c>
+      <c r="F35" t="n">
+        <v>165</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>표준-ATX</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>하단후면</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>170-200</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>case-35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>리안리 PC-O11D EVO RGB</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>미들타워</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>E-ATX;ATX;M-ATX;Mini-ITX</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>456</v>
+      </c>
+      <c r="F36" t="n">
+        <v>167</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>표준-ATX</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>하단후면</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>280/360</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>280/360</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>280/360</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11093,7 +12102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12199,6 +13208,72 @@
       <c r="D50" t="inlineStr">
         <is>
           <t>PCIe5.0x4</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ssd-50</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Micron Crucial P3 Plus M.2 NVMe 해외구매 (1TB)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>M.2 NVMe</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>PCIe4.0x4</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ssd-51</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Western Digital WD Green SN350 M.2 NVMe (1TB)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>M.2 NVMe</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>PCIe3.0x4</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ssd-52</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>삼성전자 980 M.2 NVMe (1TB)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>M.2 NVMe</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>PCIe3.0x4</t>
         </is>
       </c>
     </row>
@@ -12213,7 +13288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13099,6 +14174,96 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>cooler-air-14</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>NOCTUA NH-L9x65</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>air</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>65</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>AM4;AM5;LGA1851;LGA1700;LGA1200;LGA115x</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>{"width_mm": 95, "depth_mm": 95, "fan_size_mm": 95, "fan_count": 1, "tdp_rated_w": 84, "low_profile": true}</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>cooler-air-15</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>be quiet! DARK ROCK PRO 5</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>air</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>168</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>AM4;AM5;LGA1700;LGA1200;LGA115x</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>{"width_mm": 136, "depth_mm": 145, "fan_size_mm": 135, "fan_count": 2, "tdp_rated_w": 270}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>cooler-aio-16</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CORSAIR iCUE LINK H150i RGB</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>aqua</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>360</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>AM4;AM5;LGA2011;LGA2011-V3;LGA2066;LGA1700;LGA1200;LGA115x</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>{"radiator_length_mm": 397, "radiator_thickness_mm": 27, "fan_size_mm": 120, "fan_count": 3}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: add 8 legacy-gen parts (LGA1200/AM4 CPUs, GTX16/RX500 GPUs)
Fills the pre-RTX/RX7000 GPU gap and adds budget legacy CPUs
(i5-10400F, i3-10100F, Ryzen 7 3700X) plus matching B560/B450
boards. Only picked parts with an active danawa price -- several
older candidates (Ryzen 5 2600/2600X/3600, B460M-A, B450M DS3H)
had listings but no live sellers, so were skipped.
</commit_message>
<xml_diff>
--- a/supabase/parts_db_rebuild.xlsx
+++ b/supabase/parts_db_rebuild.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2962,6 +2962,189 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>cpu-43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>i5</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>10400F</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>코멧레이크S</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>LGA1200</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>6C/12T</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="I44" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>12MB</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>65</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>DDR4-2666</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>{"has_igpu": false}</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>cpu-44</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>i3</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>10100F</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>코멧레이크S</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>LGA1200</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>4C/8T</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I45" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>6MB</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>65</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>DDR4-2666</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>{"has_igpu": false}</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>cpu-45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>라이젠7</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>3700X</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>마티스</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>AM4</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>8C/16T</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I46" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>4MB/32MB</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>65</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>DDR4-3200</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>{"has_igpu": false}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2973,7 +3156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5744,6 +5927,120 @@
       </c>
       <c r="M50" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>mb-50</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ASRock B560M-HDV 디앤디컴</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>LGA1200</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>B560</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>M-ATX</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>244</v>
+      </c>
+      <c r="G51" t="n">
+        <v>198</v>
+      </c>
+      <c r="H51" t="n">
+        <v>1</v>
+      </c>
+      <c r="I51" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>{"pcie_x1_slots": 2, "m2_slots": 2, "sata_ports": 4, "note": "M.2 상단슬롯 세대 danawa 스펙에 명기 안 됨, B560 통상값(PCIe3.0x4)으로 추정", "source": "danawa"}</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>PCIe3.0x4</t>
+        </is>
+      </c>
+      <c r="M51" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>mb-51</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ASRock B450 스틸레전드 디앤디컴</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>AM4</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>B450</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ATX</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>305</v>
+      </c>
+      <c r="G52" t="n">
+        <v>244</v>
+      </c>
+      <c r="H52" t="n">
+        <v>2</v>
+      </c>
+      <c r="I52" t="n">
+        <v>2</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>DDR4</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>{"pcie_x1_slots": 4, "m2_slots": 2, "sata_ports": 6, "note": "M.2 상단슬롯 세대 danawa 스펙에 명기 안 됨, B450 통상값(PCIe3.0x4)으로 추정", "source": "danawa"}</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>PCIe3.0x4</t>
+        </is>
+      </c>
+      <c r="M52" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6826,7 +7123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9146,6 +9443,150 @@
       <c r="L48" t="inlineStr">
         <is>
           <t>{"boost_mhz": 2520, "pcie": "PCIe5.0x16", "stream_processors": 3584, "memory_type": "GDDR6", "source": "danawa"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>gpu-48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>GTX16</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>이엠텍 지포스 GTX 1660 SUPER MIRACLE II D6 6GB</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>6</v>
+      </c>
+      <c r="E49" t="n">
+        <v>125</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>8핀</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>450</v>
+      </c>
+      <c r="H49" t="n">
+        <v>220</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2슬롯(45mm)</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" t="b">
+        <v>1</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>{"base_mhz": 1530, "boost_mhz": 1785, "pcie": "PCIe3.0x16", "stream_processors": 1408, "memory_type": "GDDR6", "source": "danawa"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>gpu-49</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>RX500</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>액슬 라데온 RX 580 2048SP D5 8GB R2 에즈윈</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>8</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>8핀</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>500</v>
+      </c>
+      <c r="H50" t="n">
+        <v>213</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2슬롯(49mm)</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>2</v>
+      </c>
+      <c r="K50" t="b">
+        <v>1</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>{"boost_mhz": 1244, "pcie": "PCIe3.0x16", "stream_processors": 2048, "memory_type": "GDDR5", "source": "danawa"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>gpu-50</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>GTX16</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>액슬 지포스 GTX 1650 D6 4GB R3 에즈윈</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>6핀</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>300</v>
+      </c>
+      <c r="H51" t="n">
+        <v>173</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2슬롯(40mm)</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" t="b">
+        <v>1</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>{"base_mhz": 1410, "boost_mhz": 1590, "pcie": "PCIe3.0x16", "stream_processors": 896, "memory_type": "GDDR6", "source": "danawa"}</t>
         </is>
       </c>
     </row>

</xml_diff>